<commit_message>
fix: Update publications dataset with user modifications
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SmartCity20\.gemini\antigravity\scratch\surd-lab-homepage\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C3F26E-D3DC-4B3D-AEA3-9732C8DDF321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686A9505-5DA0-494C-BC72-76650D6F07B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{FB3B5A28-B30A-4FB9-B973-DA7691D44842}"/>
+    <workbookView xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21000" xr2:uid="{FB3B5A28-B30A-4FB9-B973-DA7691D44842}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -3099,10 +3099,10 @@
         <v>161</v>
       </c>
       <c r="B12" t="s">
-        <v>602</v>
+        <v>285</v>
       </c>
       <c r="C12" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D12">
         <f>VALUE(LEFT(PublicationsTable[[#This Row],[file_name]],4))</f>
@@ -3138,7 +3138,7 @@
         <v>162</v>
       </c>
       <c r="B13" t="s">
-        <v>285</v>
+        <v>602</v>
       </c>
       <c r="C13" t="s">
         <v>601</v>

</xml_diff>